<commit_message>
Azure SQL set up as code (passwordless), one setup script for Mac and Windows, call-out revenue split
- tools/database: create and lock down Azure SQL (Microsoft sign-in only, per-machine firewall, TLS 1.2,
  free serverless tier), least-privilege roles, staged all-or-nothing loads with a load log, and a
  table-by-table guide with star-schema advice and Claude MCP prompts (written to OneDrive).
- tools/setup_machine.py: one command gets the Mac or the Windows PC ready (packages, Azure CLI, git
  noreply + leak guard, OneDrive, sign-in, firewall, connection test).
- tools/githooks: stops any commit containing a password, key, data file or personal detail.
- Report builder can read the database (--source db) and prove it matches the CSVs (--compare-sources).
- Call-outs: technician time charged and materials charged (cost x 1.3) as separate revenue lines,
  ledger accounts, job columns and report numbers. Totals unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/media/exports/reports/2025-10/job-margins.xlsx
+++ b/media/exports/reports/2025-10/job-margins.xlsx
@@ -500,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D92"/>
+  <dimension ref="A1:D94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -1155,176 +1155,208 @@
         </is>
       </c>
     </row>
-    <row r="73"/>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Technician time charged, October</t>
+        </is>
+      </c>
+      <c r="B73" s="8">
+        <f>Workings!B289</f>
+        <v/>
+      </c>
+      <c r="C73" s="9" t="inlineStr">
+        <is>
+          <t>67.3% of call-out revenue</t>
+        </is>
+      </c>
+    </row>
     <row r="74">
-      <c r="A74" s="10" t="inlineStr">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Materials charged, October</t>
+        </is>
+      </c>
+      <c r="B74" s="8">
+        <f>Workings!B301</f>
+        <v/>
+      </c>
+      <c r="C74" s="9" t="inlineStr">
+        <is>
+          <t>$5,610 at cost, plus 30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="75"/>
+    <row r="76">
+      <c r="A76" s="10" t="inlineStr">
         <is>
           <t>Job gross margin on call-outs by length, October 2025</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="6" t="inlineStr"/>
-      <c r="B75" s="7" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr"/>
+      <c r="B77" s="7" t="inlineStr">
         <is>
           <t>Gross margin %</t>
         </is>
       </c>
-      <c r="C75" s="7" t="inlineStr">
+      <c r="C77" s="7" t="inlineStr">
         <is>
           <t>Gross margin $</t>
         </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>1-hour call-outs (7)</t>
-        </is>
-      </c>
-      <c r="B76" s="8">
-        <f>Workings!B288</f>
-        <v/>
-      </c>
-      <c r="C76" s="11">
-        <f>Workings!B287</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>1.5-hour call-outs (3)</t>
-        </is>
-      </c>
-      <c r="B77" s="8">
-        <f>Workings!B299</f>
-        <v/>
-      </c>
-      <c r="C77" s="11">
-        <f>Workings!B298</f>
-        <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2-hour call-outs (9)</t>
+          <t>1-hour call-outs (7)</t>
         </is>
       </c>
       <c r="B78" s="8">
-        <f>Workings!B310</f>
+        <f>Workings!B314</f>
         <v/>
       </c>
       <c r="C78" s="11">
-        <f>Workings!B309</f>
+        <f>Workings!B313</f>
         <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2.5-hour call-outs (8)</t>
+          <t>1.5-hour call-outs (3)</t>
         </is>
       </c>
       <c r="B79" s="8">
-        <f>Workings!B321</f>
+        <f>Workings!B327</f>
         <v/>
       </c>
       <c r="C79" s="11">
-        <f>Workings!B320</f>
+        <f>Workings!B326</f>
         <v/>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>3-hour call-outs (10)</t>
+          <t>2-hour call-outs (9)</t>
         </is>
       </c>
       <c r="B80" s="8">
-        <f>Workings!B332</f>
+        <f>Workings!B340</f>
         <v/>
       </c>
       <c r="C80" s="11">
-        <f>Workings!B331</f>
+        <f>Workings!B339</f>
         <v/>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
+          <t>2.5-hour call-outs (8)</t>
+        </is>
+      </c>
+      <c r="B81" s="8">
+        <f>Workings!B353</f>
+        <v/>
+      </c>
+      <c r="C81" s="11">
+        <f>Workings!B352</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>3-hour call-outs (10)</t>
+        </is>
+      </c>
+      <c r="B82" s="8">
+        <f>Workings!B366</f>
+        <v/>
+      </c>
+      <c r="C82" s="11">
+        <f>Workings!B365</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
           <t>4-hour call-outs (6)</t>
         </is>
       </c>
-      <c r="B81" s="8">
-        <f>Workings!B343</f>
-        <v/>
-      </c>
-      <c r="C81" s="11">
-        <f>Workings!B342</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82"/>
-    <row r="83">
-      <c r="A83" s="4" t="inlineStr">
+      <c r="B83" s="8">
+        <f>Workings!B379</f>
+        <v/>
+      </c>
+      <c r="C83" s="11">
+        <f>Workings!B378</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84"/>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
         <is>
           <t>What it shows</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="45" customHeight="1">
-      <c r="A84" s="3" t="inlineStr">
-        <is>
-          <t>43 call-outs in October made a 43.3% job gross margin between them. Gross margins run from 37.8% to 45.9% by length: the hourly rate covers technician time comfortably, so the gross margin mostly moves with how much material goes on the van.</t>
-        </is>
-      </c>
-    </row>
-    <row r="85"/>
-    <row r="86">
-      <c r="A86" s="4" t="inlineStr">
+    <row r="86" ht="60" customHeight="1">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>43 call-outs in October billed $15,005 of technician time and $7,293 of materials ($5,610 at cost plus 30%), and made a 43.3% job gross margin between them. Gross margins run from 37.8% to 45.9% by length: the hourly rate covers technician time comfortably, so the gross margin mostly moves with how much material goes on the van.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87"/>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
         <is>
           <t>What you'd do about it</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="30" customHeight="1">
-      <c r="A87" s="3" t="inlineStr">
+    <row r="89" ht="30" customHeight="1">
+      <c r="A89" s="3" t="inlineStr">
         <is>
           <t>Call-outs: 43.3% gross margin, below the 52.5% needed to cover overheads.</t>
         </is>
       </c>
     </row>
-    <row r="88"/>
-    <row r="89">
-      <c r="A89" s="5" t="inlineStr">
+    <row r="90"/>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
         <is>
           <t>Every type of job at once</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="12" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="12" t="inlineStr">
         <is>
           <t>Job gross margin by month: every month is on the Data sheet.</t>
         </is>
       </c>
     </row>
-    <row r="91"/>
-    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A89:D89"/>
     <mergeCell ref="A68:D68"/>
+    <mergeCell ref="A86:D86"/>
     <mergeCell ref="A52:D52"/>
-    <mergeCell ref="A87:D87"/>
     <mergeCell ref="A65:D65"/>
     <mergeCell ref="A24:D24"/>
     <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A84:D84"/>
     <mergeCell ref="A49:D49"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
@@ -1352,7 +1384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C346"/>
+  <dimension ref="A1:C382"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -3676,14 +3708,14 @@
     <row r="280">
       <c r="A280" s="5" t="inlineStr">
         <is>
-          <t>1-hour call-outs (7)</t>
+          <t>Call-out revenue, October</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="12" t="inlineStr">
         <is>
-          <t>Call-outs of this length in October, added together</t>
+          <t>Technician time charged at $145/hour + materials charged at cost × 1.3</t>
         </is>
       </c>
     </row>
@@ -3698,498 +3730,818 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Call-outs</t>
+          <t>Technician time charged ($145/hour)</t>
         </is>
       </c>
       <c r="B283" s="13" t="n">
-        <v>7</v>
+        <v>15005</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Materials at cost</t>
         </is>
       </c>
       <c r="B284" s="13" t="n">
-        <v>2068</v>
+        <v>5610</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="B285" s="13" t="n">
-        <v>-810</v>
+          <t>Mark-up on materials</t>
+        </is>
+      </c>
+      <c r="B285" s="14" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Technician time at cost</t>
-        </is>
-      </c>
-      <c r="B286" s="13" t="n">
-        <v>-476</v>
+          <t>Materials charged (cost × 1.3)</t>
+        </is>
+      </c>
+      <c r="B286" s="13">
+        <f>B284*(1+B285)</f>
+        <v/>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Job gross margin</t>
-        </is>
-      </c>
-      <c r="B287" s="13">
-        <f>B284+B285+B286</f>
-        <v/>
+          <t>Materials charged (as invoiced, rounded per call-out)</t>
+        </is>
+      </c>
+      <c r="B287" s="13" t="n">
+        <v>7293</v>
       </c>
     </row>
     <row r="288">
-      <c r="A288" s="15" t="inlineStr">
-        <is>
-          <t>Job gross margin %</t>
-        </is>
-      </c>
-      <c r="B288" s="16">
-        <f>B287/B284</f>
-        <v/>
-      </c>
-    </row>
-    <row r="289"/>
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Call-out revenue</t>
+        </is>
+      </c>
+      <c r="B288" s="13">
+        <f>B283+B287</f>
+        <v/>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="15" t="inlineStr">
+        <is>
+          <t>Technician time, % of call-out revenue</t>
+        </is>
+      </c>
+      <c r="B289" s="16">
+        <f>B283/B288</f>
+        <v/>
+      </c>
+    </row>
     <row r="290"/>
-    <row r="291">
-      <c r="A291" s="5" t="inlineStr">
-        <is>
-          <t>1.5-hour call-outs (3)</t>
-        </is>
-      </c>
-    </row>
+    <row r="291"/>
     <row r="292">
-      <c r="A292" s="12" t="inlineStr">
-        <is>
-          <t>Call-outs of this length in October, added together</t>
+      <c r="A292" s="5" t="inlineStr">
+        <is>
+          <t>Call-out revenue, October</t>
         </is>
       </c>
     </row>
     <row r="293">
-      <c r="A293" s="6" t="inlineStr"/>
-      <c r="B293" s="7" t="inlineStr">
+      <c r="A293" s="12" t="inlineStr">
+        <is>
+          <t>Technician time charged at $145/hour + materials charged at cost × 1.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="6" t="inlineStr"/>
+      <c r="B294" s="7" t="inlineStr">
         <is>
           <t>Oct 2025</t>
         </is>
-      </c>
-    </row>
-    <row r="294">
-      <c r="A294" t="inlineStr">
-        <is>
-          <t>Call-outs</t>
-        </is>
-      </c>
-      <c r="B294" s="13" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>Revenue</t>
+          <t>Technician time charged ($145/hour)</t>
         </is>
       </c>
       <c r="B295" s="13" t="n">
-        <v>1288</v>
+        <v>15005</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Materials at cost</t>
         </is>
       </c>
       <c r="B296" s="13" t="n">
-        <v>-490</v>
+        <v>5610</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>Technician time at cost</t>
-        </is>
-      </c>
-      <c r="B297" s="13" t="n">
-        <v>-306</v>
+          <t>Mark-up on materials</t>
+        </is>
+      </c>
+      <c r="B297" s="14" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>Job gross margin</t>
+          <t>Materials charged (cost × 1.3)</t>
         </is>
       </c>
       <c r="B298" s="13">
-        <f>B295+B296+B297</f>
+        <f>B296*(1+B297)</f>
         <v/>
       </c>
     </row>
     <row r="299">
-      <c r="A299" s="15" t="inlineStr">
-        <is>
-          <t>Job gross margin %</t>
-        </is>
-      </c>
-      <c r="B299" s="16">
-        <f>B298/B295</f>
-        <v/>
-      </c>
-    </row>
-    <row r="300"/>
-    <row r="301"/>
-    <row r="302">
-      <c r="A302" s="5" t="inlineStr">
-        <is>
-          <t>2-hour call-outs (9)</t>
-        </is>
-      </c>
-    </row>
-    <row r="303">
-      <c r="A303" s="12" t="inlineStr">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Materials charged (as invoiced, rounded per call-out)</t>
+        </is>
+      </c>
+      <c r="B299" s="13" t="n">
+        <v>7293</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Call-out revenue</t>
+        </is>
+      </c>
+      <c r="B300" s="13">
+        <f>B295+B299</f>
+        <v/>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="15" t="inlineStr">
+        <is>
+          <t>Technician time, % of call-out revenue</t>
+        </is>
+      </c>
+      <c r="B301" s="16">
+        <f>B295/B300</f>
+        <v/>
+      </c>
+    </row>
+    <row r="302"/>
+    <row r="303"/>
+    <row r="304">
+      <c r="A304" s="5" t="inlineStr">
+        <is>
+          <t>1-hour call-outs (7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="12" t="inlineStr">
         <is>
           <t>Call-outs of this length in October, added together</t>
         </is>
       </c>
     </row>
-    <row r="304">
-      <c r="A304" s="6" t="inlineStr"/>
-      <c r="B304" s="7" t="inlineStr">
+    <row r="306">
+      <c r="A306" s="6" t="inlineStr"/>
+      <c r="B306" s="7" t="inlineStr">
         <is>
           <t>Oct 2025</t>
         </is>
-      </c>
-    </row>
-    <row r="305">
-      <c r="A305" t="inlineStr">
-        <is>
-          <t>Call-outs</t>
-        </is>
-      </c>
-      <c r="B305" s="13" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="306">
-      <c r="A306" t="inlineStr">
-        <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="B306" s="13" t="n">
-        <v>4443</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Call-outs</t>
         </is>
       </c>
       <c r="B307" s="13" t="n">
-        <v>-1410</v>
+        <v>7</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>Technician time at cost</t>
+          <t>Technician time charged ($145/hour)</t>
         </is>
       </c>
       <c r="B308" s="13" t="n">
-        <v>-1224</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
+          <t>Materials charged (cost × 1.3)</t>
+        </is>
+      </c>
+      <c r="B309" s="13" t="n">
+        <v>1053</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B310" s="13">
+        <f>B308+B309</f>
+        <v/>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Materials at cost</t>
+        </is>
+      </c>
+      <c r="B311" s="13" t="n">
+        <v>-810</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Technician time at cost</t>
+        </is>
+      </c>
+      <c r="B312" s="13" t="n">
+        <v>-476</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
           <t>Job gross margin</t>
         </is>
       </c>
-      <c r="B309" s="13">
-        <f>B306+B307+B308</f>
-        <v/>
-      </c>
-    </row>
-    <row r="310">
-      <c r="A310" s="15" t="inlineStr">
+      <c r="B313" s="13">
+        <f>B310+B311+B312</f>
+        <v/>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="15" t="inlineStr">
         <is>
           <t>Job gross margin %</t>
         </is>
       </c>
-      <c r="B310" s="16">
-        <f>B309/B306</f>
-        <v/>
-      </c>
-    </row>
-    <row r="311"/>
-    <row r="312"/>
-    <row r="313">
-      <c r="A313" s="5" t="inlineStr">
-        <is>
-          <t>2.5-hour call-outs (8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="314">
-      <c r="A314" s="12" t="inlineStr">
+      <c r="B314" s="16">
+        <f>B313/B310</f>
+        <v/>
+      </c>
+    </row>
+    <row r="315"/>
+    <row r="316"/>
+    <row r="317">
+      <c r="A317" s="5" t="inlineStr">
+        <is>
+          <t>1.5-hour call-outs (3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="12" t="inlineStr">
         <is>
           <t>Call-outs of this length in October, added together</t>
         </is>
       </c>
     </row>
-    <row r="315">
-      <c r="A315" s="6" t="inlineStr"/>
-      <c r="B315" s="7" t="inlineStr">
+    <row r="319">
+      <c r="A319" s="6" t="inlineStr"/>
+      <c r="B319" s="7" t="inlineStr">
         <is>
           <t>Oct 2025</t>
         </is>
-      </c>
-    </row>
-    <row r="316">
-      <c r="A316" t="inlineStr">
-        <is>
-          <t>Call-outs</t>
-        </is>
-      </c>
-      <c r="B316" s="13" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="317">
-      <c r="A317" t="inlineStr">
-        <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="B317" s="13" t="n">
-        <v>4134</v>
-      </c>
-    </row>
-    <row r="318">
-      <c r="A318" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="B318" s="13" t="n">
-        <v>-950</v>
-      </c>
-    </row>
-    <row r="319">
-      <c r="A319" t="inlineStr">
-        <is>
-          <t>Technician time at cost</t>
-        </is>
-      </c>
-      <c r="B319" s="13" t="n">
-        <v>-1360</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
+          <t>Call-outs</t>
+        </is>
+      </c>
+      <c r="B320" s="13" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Technician time charged ($145/hour)</t>
+        </is>
+      </c>
+      <c r="B321" s="13" t="n">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Materials charged (cost × 1.3)</t>
+        </is>
+      </c>
+      <c r="B322" s="13" t="n">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B323" s="13">
+        <f>B321+B322</f>
+        <v/>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Materials at cost</t>
+        </is>
+      </c>
+      <c r="B324" s="13" t="n">
+        <v>-490</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Technician time at cost</t>
+        </is>
+      </c>
+      <c r="B325" s="13" t="n">
+        <v>-306</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
           <t>Job gross margin</t>
         </is>
       </c>
-      <c r="B320" s="13">
-        <f>B317+B318+B319</f>
-        <v/>
-      </c>
-    </row>
-    <row r="321">
-      <c r="A321" s="15" t="inlineStr">
+      <c r="B326" s="13">
+        <f>B323+B324+B325</f>
+        <v/>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="15" t="inlineStr">
         <is>
           <t>Job gross margin %</t>
         </is>
       </c>
-      <c r="B321" s="16">
-        <f>B320/B317</f>
-        <v/>
-      </c>
-    </row>
-    <row r="322"/>
-    <row r="323"/>
-    <row r="324">
-      <c r="A324" s="5" t="inlineStr">
-        <is>
-          <t>3-hour call-outs (10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="325">
-      <c r="A325" s="12" t="inlineStr">
+      <c r="B327" s="16">
+        <f>B326/B323</f>
+        <v/>
+      </c>
+    </row>
+    <row r="328"/>
+    <row r="329"/>
+    <row r="330">
+      <c r="A330" s="5" t="inlineStr">
+        <is>
+          <t>2-hour call-outs (9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="12" t="inlineStr">
         <is>
           <t>Call-outs of this length in October, added together</t>
         </is>
       </c>
     </row>
-    <row r="326">
-      <c r="A326" s="6" t="inlineStr"/>
-      <c r="B326" s="7" t="inlineStr">
+    <row r="332">
+      <c r="A332" s="6" t="inlineStr"/>
+      <c r="B332" s="7" t="inlineStr">
         <is>
           <t>Oct 2025</t>
         </is>
       </c>
     </row>
-    <row r="327">
-      <c r="A327" t="inlineStr">
+    <row r="333">
+      <c r="A333" t="inlineStr">
         <is>
           <t>Call-outs</t>
         </is>
       </c>
-      <c r="B327" s="13" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="328">
-      <c r="A328" t="inlineStr">
+      <c r="B333" s="13" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Technician time charged ($145/hour)</t>
+        </is>
+      </c>
+      <c r="B334" s="13" t="n">
+        <v>2610</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Materials charged (cost × 1.3)</t>
+        </is>
+      </c>
+      <c r="B335" s="13" t="n">
+        <v>1833</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B328" s="13" t="n">
-        <v>5780</v>
-      </c>
-    </row>
-    <row r="329">
-      <c r="A329" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="B329" s="13" t="n">
-        <v>-1100</v>
-      </c>
-    </row>
-    <row r="330">
-      <c r="A330" t="inlineStr">
-        <is>
-          <t>Technician time at cost</t>
-        </is>
-      </c>
-      <c r="B330" s="13" t="n">
-        <v>-2040</v>
-      </c>
-    </row>
-    <row r="331">
-      <c r="A331" t="inlineStr">
-        <is>
-          <t>Job gross margin</t>
-        </is>
-      </c>
-      <c r="B331" s="13">
-        <f>B328+B329+B330</f>
-        <v/>
-      </c>
-    </row>
-    <row r="332">
-      <c r="A332" s="15" t="inlineStr">
-        <is>
-          <t>Job gross margin %</t>
-        </is>
-      </c>
-      <c r="B332" s="16">
-        <f>B331/B328</f>
-        <v/>
-      </c>
-    </row>
-    <row r="333"/>
-    <row r="334"/>
-    <row r="335">
-      <c r="A335" s="5" t="inlineStr">
-        <is>
-          <t>4-hour call-outs (6)</t>
-        </is>
-      </c>
-    </row>
-    <row r="336">
-      <c r="A336" s="12" t="inlineStr">
-        <is>
-          <t>Call-outs of this length in October, added together</t>
-        </is>
+      <c r="B336" s="13">
+        <f>B334+B335</f>
+        <v/>
       </c>
     </row>
     <row r="337">
-      <c r="A337" s="6" t="inlineStr"/>
-      <c r="B337" s="7" t="inlineStr">
-        <is>
-          <t>Oct 2025</t>
-        </is>
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Materials at cost</t>
+        </is>
+      </c>
+      <c r="B337" s="13" t="n">
+        <v>-1410</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>Call-outs</t>
+          <t>Technician time at cost</t>
         </is>
       </c>
       <c r="B338" s="13" t="n">
-        <v>6</v>
+        <v>-1224</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
+          <t>Job gross margin</t>
+        </is>
+      </c>
+      <c r="B339" s="13">
+        <f>B336+B337+B338</f>
+        <v/>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="15" t="inlineStr">
+        <is>
+          <t>Job gross margin %</t>
+        </is>
+      </c>
+      <c r="B340" s="16">
+        <f>B339/B336</f>
+        <v/>
+      </c>
+    </row>
+    <row r="341"/>
+    <row r="342"/>
+    <row r="343">
+      <c r="A343" s="5" t="inlineStr">
+        <is>
+          <t>2.5-hour call-outs (8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="12" t="inlineStr">
+        <is>
+          <t>Call-outs of this length in October, added together</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="6" t="inlineStr"/>
+      <c r="B345" s="7" t="inlineStr">
+        <is>
+          <t>Oct 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Call-outs</t>
+        </is>
+      </c>
+      <c r="B346" s="13" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>Technician time charged ($145/hour)</t>
+        </is>
+      </c>
+      <c r="B347" s="13" t="n">
+        <v>2899</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>Materials charged (cost × 1.3)</t>
+        </is>
+      </c>
+      <c r="B348" s="13" t="n">
+        <v>1235</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B339" s="13" t="n">
-        <v>4585</v>
-      </c>
-    </row>
-    <row r="340">
-      <c r="A340" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="B340" s="13" t="n">
+      <c r="B349" s="13">
+        <f>B347+B348</f>
+        <v/>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Materials at cost</t>
+        </is>
+      </c>
+      <c r="B350" s="13" t="n">
+        <v>-950</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>Technician time at cost</t>
+        </is>
+      </c>
+      <c r="B351" s="13" t="n">
+        <v>-1360</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>Job gross margin</t>
+        </is>
+      </c>
+      <c r="B352" s="13">
+        <f>B349+B350+B351</f>
+        <v/>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="15" t="inlineStr">
+        <is>
+          <t>Job gross margin %</t>
+        </is>
+      </c>
+      <c r="B353" s="16">
+        <f>B352/B349</f>
+        <v/>
+      </c>
+    </row>
+    <row r="354"/>
+    <row r="355"/>
+    <row r="356">
+      <c r="A356" s="5" t="inlineStr">
+        <is>
+          <t>3-hour call-outs (10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="12" t="inlineStr">
+        <is>
+          <t>Call-outs of this length in October, added together</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="6" t="inlineStr"/>
+      <c r="B358" s="7" t="inlineStr">
+        <is>
+          <t>Oct 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>Call-outs</t>
+        </is>
+      </c>
+      <c r="B359" s="13" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>Technician time charged ($145/hour)</t>
+        </is>
+      </c>
+      <c r="B360" s="13" t="n">
+        <v>4350</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>Materials charged (cost × 1.3)</t>
+        </is>
+      </c>
+      <c r="B361" s="13" t="n">
+        <v>1430</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B362" s="13">
+        <f>B360+B361</f>
+        <v/>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>Materials at cost</t>
+        </is>
+      </c>
+      <c r="B363" s="13" t="n">
+        <v>-1100</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>Technician time at cost</t>
+        </is>
+      </c>
+      <c r="B364" s="13" t="n">
+        <v>-2040</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>Job gross margin</t>
+        </is>
+      </c>
+      <c r="B365" s="13">
+        <f>B362+B363+B364</f>
+        <v/>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="15" t="inlineStr">
+        <is>
+          <t>Job gross margin %</t>
+        </is>
+      </c>
+      <c r="B366" s="16">
+        <f>B365/B362</f>
+        <v/>
+      </c>
+    </row>
+    <row r="367"/>
+    <row r="368"/>
+    <row r="369">
+      <c r="A369" s="5" t="inlineStr">
+        <is>
+          <t>4-hour call-outs (6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="12" t="inlineStr">
+        <is>
+          <t>Call-outs of this length in October, added together</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="6" t="inlineStr"/>
+      <c r="B371" s="7" t="inlineStr">
+        <is>
+          <t>Oct 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>Call-outs</t>
+        </is>
+      </c>
+      <c r="B372" s="13" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>Technician time charged ($145/hour)</t>
+        </is>
+      </c>
+      <c r="B373" s="13" t="n">
+        <v>3480</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>Materials charged (cost × 1.3)</t>
+        </is>
+      </c>
+      <c r="B374" s="13" t="n">
+        <v>1105</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B375" s="13">
+        <f>B373+B374</f>
+        <v/>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>Materials at cost</t>
+        </is>
+      </c>
+      <c r="B376" s="13" t="n">
         <v>-850</v>
       </c>
     </row>
-    <row r="341">
-      <c r="A341" t="inlineStr">
+    <row r="377">
+      <c r="A377" t="inlineStr">
         <is>
           <t>Technician time at cost</t>
         </is>
       </c>
-      <c r="B341" s="13" t="n">
+      <c r="B377" s="13" t="n">
         <v>-1632</v>
       </c>
     </row>
-    <row r="342">
-      <c r="A342" t="inlineStr">
+    <row r="378">
+      <c r="A378" t="inlineStr">
         <is>
           <t>Job gross margin</t>
         </is>
       </c>
-      <c r="B342" s="13">
-        <f>B339+B340+B341</f>
-        <v/>
-      </c>
-    </row>
-    <row r="343">
-      <c r="A343" s="15" t="inlineStr">
+      <c r="B378" s="13">
+        <f>B375+B376+B377</f>
+        <v/>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="15" t="inlineStr">
         <is>
           <t>Job gross margin %</t>
         </is>
       </c>
-      <c r="B343" s="16">
-        <f>B342/B339</f>
-        <v/>
-      </c>
-    </row>
-    <row r="344"/>
-    <row r="345"/>
-    <row r="346"/>
+      <c r="B379" s="16">
+        <f>B378/B375</f>
+        <v/>
+      </c>
+    </row>
+    <row r="380"/>
+    <row r="381"/>
+    <row r="382"/>
   </sheetData>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.5" footer="0.5"/>
@@ -4202,7 +4554,7 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <rowBreaks count="13" manualBreakCount="13">
+  <rowBreaks count="14" manualBreakCount="14">
     <brk id="30" min="0" max="16383" man="1"/>
     <brk id="57" min="0" max="16383" man="1"/>
     <brk id="79" min="0" max="16383" man="1"/>
@@ -4214,8 +4566,9 @@
     <brk id="231" min="0" max="16383" man="1"/>
     <brk id="257" min="0" max="16383" man="1"/>
     <brk id="279" min="0" max="16383" man="1"/>
-    <brk id="301" min="0" max="16383" man="1"/>
-    <brk id="323" min="0" max="16383" man="1"/>
+    <brk id="303" min="0" max="16383" man="1"/>
+    <brk id="329" min="0" max="16383" man="1"/>
+    <brk id="355" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Excel: target and break-even drawn as vertical lines on bar charts (bar + XY scatter combo on hidden secondary axes), checked in Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/media/exports/reports/2025-10/job-margins.xlsx
+++ b/media/exports/reports/2025-10/job-margins.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart lines" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="Job_gross_margin_October_All_jobs">'Report'!$B$15</definedName>
@@ -28,8 +29,8 @@
     <definedName name="Materials_charged_October">'Report'!$B$107</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$D$132</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Workings'!$A$1:$C$483</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Data'!$5:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Data'!$A$1:$G$57</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Data'!$5:$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Data'!$A$1:$G$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -264,7 +265,7 @@
                 </a:solidFill>
                 <a:latin typeface="Roboto"/>
               </a:rPr>
-              <a:t>Job gross margin by type of job, October 2025 · target 35.0%</a:t>
+              <a:t>Job gross margin by type of job, October 2025</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -331,6 +332,154 @@
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
+      <scatterChart>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Target 35.0%</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="25342A"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <dLbl>
+              <idx val="1"/>
+              <txPr>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                  <a:pPr>
+                    <a:defRPr sz="900" b="1">
+                      <a:solidFill>
+                        <a:srgbClr val="25342A"/>
+                      </a:solidFill>
+                      <a:latin typeface="Roboto"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:r>
+                    <a:t/>
+                  </a:r>
+                  <a:endParaRPr sz="900" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="25342A"/>
+                    </a:solidFill>
+                    <a:latin typeface="Roboto"/>
+                  </a:endParaRPr>
+                </a:p>
+              </txPr>
+              <dLblPos val="r"/>
+              <showLegendKey val="0"/>
+              <showVal val="0"/>
+              <showCatName val="0"/>
+              <showSerName val="1"/>
+              <showPercent val="0"/>
+            </dLbl>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
+          <xVal>
+            <numRef>
+              <f>'Chart lines'!$B$4:$B$5</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Chart lines'!$C$4:$C$5</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>Break-even 52.5%</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="B42318"/>
+              </a:solidFill>
+              <a:prstDash val="sysDot"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <dLbl>
+              <idx val="1"/>
+              <txPr>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                  <a:pPr>
+                    <a:defRPr sz="900" b="1">
+                      <a:solidFill>
+                        <a:srgbClr val="B42318"/>
+                      </a:solidFill>
+                      <a:latin typeface="Roboto"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:r>
+                    <a:t/>
+                  </a:r>
+                  <a:endParaRPr sz="900" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="B42318"/>
+                    </a:solidFill>
+                    <a:latin typeface="Roboto"/>
+                  </a:endParaRPr>
+                </a:p>
+              </txPr>
+              <dLblPos val="l"/>
+              <showLegendKey val="0"/>
+              <showVal val="0"/>
+              <showCatName val="0"/>
+              <showSerName val="1"/>
+              <showPercent val="0"/>
+            </dLbl>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
+          <xVal>
+            <numRef>
+              <f>'Chart lines'!$B$8:$B$9</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Chart lines'!$C$8:$C$9</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <axId val="500"/>
+        <axId val="600"/>
+      </scatterChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -346,6 +495,8 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="0.6842499999999999"/>
+          <min val="0"/>
         </scaling>
         <delete val="1"/>
         <axPos val="l"/>
@@ -353,6 +504,33 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+      </valAx>
+      <valAx>
+        <axId val="500"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="0.6842499999999999"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="t"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="600"/>
+      </valAx>
+      <valAx>
+        <axId val="600"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="1.08"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="r"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="500"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -385,7 +563,7 @@
                 </a:solidFill>
                 <a:latin typeface="Roboto"/>
               </a:rPr>
-              <a:t>Job gross margin on each maintenance contract, October 2025 · target 35.0%</a:t>
+              <a:t>Job gross margin on each maintenance contract, October 2025</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -438,6 +616,154 @@
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
+      <scatterChart>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Target 35.0%</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="25342A"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <dLbl>
+              <idx val="1"/>
+              <txPr>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                  <a:pPr>
+                    <a:defRPr sz="900" b="1">
+                      <a:solidFill>
+                        <a:srgbClr val="25342A"/>
+                      </a:solidFill>
+                      <a:latin typeface="Roboto"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:r>
+                    <a:t/>
+                  </a:r>
+                  <a:endParaRPr sz="900" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="25342A"/>
+                    </a:solidFill>
+                    <a:latin typeface="Roboto"/>
+                  </a:endParaRPr>
+                </a:p>
+              </txPr>
+              <dLblPos val="r"/>
+              <showLegendKey val="0"/>
+              <showVal val="0"/>
+              <showCatName val="0"/>
+              <showSerName val="1"/>
+              <showPercent val="0"/>
+            </dLbl>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
+          <xVal>
+            <numRef>
+              <f>'Chart lines'!$B$12:$B$13</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Chart lines'!$C$12:$C$13</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>Break-even 52.5%</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="B42318"/>
+              </a:solidFill>
+              <a:prstDash val="sysDot"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <dLbl>
+              <idx val="1"/>
+              <txPr>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                  <a:pPr>
+                    <a:defRPr sz="900" b="1">
+                      <a:solidFill>
+                        <a:srgbClr val="B42318"/>
+                      </a:solidFill>
+                      <a:latin typeface="Roboto"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:r>
+                    <a:t/>
+                  </a:r>
+                  <a:endParaRPr sz="900" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="B42318"/>
+                    </a:solidFill>
+                    <a:latin typeface="Roboto"/>
+                  </a:endParaRPr>
+                </a:p>
+              </txPr>
+              <dLblPos val="l"/>
+              <showLegendKey val="0"/>
+              <showVal val="0"/>
+              <showCatName val="0"/>
+              <showSerName val="1"/>
+              <showPercent val="0"/>
+            </dLbl>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
+          <xVal>
+            <numRef>
+              <f>'Chart lines'!$B$16:$B$17</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Chart lines'!$C$16:$C$17</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <axId val="500"/>
+        <axId val="600"/>
+      </scatterChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -453,6 +779,8 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="0.7026499999999999"/>
+          <min val="0"/>
         </scaling>
         <delete val="1"/>
         <axPos val="l"/>
@@ -460,6 +788,33 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+      </valAx>
+      <valAx>
+        <axId val="500"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="0.7026499999999999"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="t"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="600"/>
+      </valAx>
+      <valAx>
+        <axId val="600"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="1.08"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="r"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="500"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -492,7 +847,7 @@
                 </a:solidFill>
                 <a:latin typeface="Roboto"/>
               </a:rPr>
-              <a:t>Job gross margin on each installation invoiced in October 2025 · target 35.0%</a:t>
+              <a:t>Job gross margin on each installation invoiced in October 2025</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -573,6 +928,154 @@
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
+      <scatterChart>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Target 35.0%</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="25342A"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <dLbl>
+              <idx val="1"/>
+              <txPr>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                  <a:pPr>
+                    <a:defRPr sz="900" b="1">
+                      <a:solidFill>
+                        <a:srgbClr val="25342A"/>
+                      </a:solidFill>
+                      <a:latin typeface="Roboto"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:r>
+                    <a:t/>
+                  </a:r>
+                  <a:endParaRPr sz="900" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="25342A"/>
+                    </a:solidFill>
+                    <a:latin typeface="Roboto"/>
+                  </a:endParaRPr>
+                </a:p>
+              </txPr>
+              <dLblPos val="r"/>
+              <showLegendKey val="0"/>
+              <showVal val="0"/>
+              <showCatName val="0"/>
+              <showSerName val="1"/>
+              <showPercent val="0"/>
+            </dLbl>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
+          <xVal>
+            <numRef>
+              <f>'Chart lines'!$B$20:$B$21</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Chart lines'!$C$20:$C$21</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>Break-even 52.5%</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="B42318"/>
+              </a:solidFill>
+              <a:prstDash val="sysDot"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <dLbl>
+              <idx val="1"/>
+              <txPr>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                  <a:pPr>
+                    <a:defRPr sz="900" b="1">
+                      <a:solidFill>
+                        <a:srgbClr val="B42318"/>
+                      </a:solidFill>
+                      <a:latin typeface="Roboto"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:r>
+                    <a:t/>
+                  </a:r>
+                  <a:endParaRPr sz="900" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="B42318"/>
+                    </a:solidFill>
+                    <a:latin typeface="Roboto"/>
+                  </a:endParaRPr>
+                </a:p>
+              </txPr>
+              <dLblPos val="l"/>
+              <showLegendKey val="0"/>
+              <showVal val="0"/>
+              <showCatName val="0"/>
+              <showSerName val="1"/>
+              <showPercent val="0"/>
+            </dLbl>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
+          <xVal>
+            <numRef>
+              <f>'Chart lines'!$B$24:$B$25</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Chart lines'!$C$24:$C$25</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <axId val="500"/>
+        <axId val="600"/>
+      </scatterChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -588,6 +1091,8 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="0.60375"/>
+          <min val="0"/>
         </scaling>
         <delete val="1"/>
         <axPos val="l"/>
@@ -595,6 +1100,33 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+      </valAx>
+      <valAx>
+        <axId val="500"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="0.60375"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="t"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="600"/>
+      </valAx>
+      <valAx>
+        <axId val="600"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="1.08"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="r"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="500"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -627,7 +1159,7 @@
                 </a:solidFill>
                 <a:latin typeface="Roboto"/>
               </a:rPr>
-              <a:t>Job gross margin on call-outs by length, October 2025 · target 35.0%</a:t>
+              <a:t>Job gross margin on call-outs by length, October 2025</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -680,6 +1212,154 @@
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
+      <scatterChart>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Target 35.0%</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="25342A"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <dLbl>
+              <idx val="1"/>
+              <txPr>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                  <a:pPr>
+                    <a:defRPr sz="900" b="1">
+                      <a:solidFill>
+                        <a:srgbClr val="25342A"/>
+                      </a:solidFill>
+                      <a:latin typeface="Roboto"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:r>
+                    <a:t/>
+                  </a:r>
+                  <a:endParaRPr sz="900" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="25342A"/>
+                    </a:solidFill>
+                    <a:latin typeface="Roboto"/>
+                  </a:endParaRPr>
+                </a:p>
+              </txPr>
+              <dLblPos val="r"/>
+              <showLegendKey val="0"/>
+              <showVal val="0"/>
+              <showCatName val="0"/>
+              <showSerName val="1"/>
+              <showPercent val="0"/>
+            </dLbl>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
+          <xVal>
+            <numRef>
+              <f>'Chart lines'!$B$28:$B$29</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Chart lines'!$C$28:$C$29</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>Break-even 52.5%</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="B42318"/>
+              </a:solidFill>
+              <a:prstDash val="sysDot"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <dLbl>
+              <idx val="1"/>
+              <txPr>
+                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                  <a:pPr>
+                    <a:defRPr sz="900" b="1">
+                      <a:solidFill>
+                        <a:srgbClr val="B42318"/>
+                      </a:solidFill>
+                      <a:latin typeface="Roboto"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:r>
+                    <a:t/>
+                  </a:r>
+                  <a:endParaRPr sz="900" b="1">
+                    <a:solidFill>
+                      <a:srgbClr val="B42318"/>
+                    </a:solidFill>
+                    <a:latin typeface="Roboto"/>
+                  </a:endParaRPr>
+                </a:p>
+              </txPr>
+              <dLblPos val="l"/>
+              <showLegendKey val="0"/>
+              <showVal val="0"/>
+              <showCatName val="0"/>
+              <showSerName val="1"/>
+              <showPercent val="0"/>
+            </dLbl>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
+          <xVal>
+            <numRef>
+              <f>'Chart lines'!$B$32:$B$33</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Chart lines'!$C$32:$C$33</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <axId val="500"/>
+        <axId val="600"/>
+      </scatterChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -695,6 +1375,8 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="0.60375"/>
+          <min val="0"/>
         </scaling>
         <delete val="1"/>
         <axPos val="l"/>
@@ -702,6 +1384,33 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+      </valAx>
+      <valAx>
+        <axId val="500"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="0.60375"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="t"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="600"/>
+      </valAx>
+      <valAx>
+        <axId val="600"/>
+        <scaling>
+          <orientation val="minMax"/>
+          <max val="1.08"/>
+          <min val="0"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="r"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="500"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -927,7 +1636,7 @@
       <row>19</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="1980000"/>
+    <ext cx="5400000" cy="2196000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -949,7 +1658,7 @@
       <row>45</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="3960000"/>
+    <ext cx="5400000" cy="4176000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -971,7 +1680,7 @@
       <row>81</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="1980000"/>
+    <ext cx="5400000" cy="2196000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="3" name="Chart 3"/>
@@ -993,7 +1702,7 @@
       <row>109</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="2340000"/>
+    <ext cx="5400000" cy="2556000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="4" name="Chart 4"/>
@@ -1369,7 +2078,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Period: October 2025 · Data status: Sep 2025 locked · Oct 2025 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:35am</t>
+          <t>Period: October 2025 · Data status: Sep 2025 locked · Oct 2025 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 10:11am</t>
         </is>
       </c>
     </row>
@@ -2367,7 +3076,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Electrical &amp;&amp; Air Pty Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 job-margins.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:35am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 job-margins.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 10:11am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2416,7 +3125,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Period: October 2025 · Data status: Sep 2025 locked · Oct 2025 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:35am</t>
+          <t>Period: October 2025 · Data status: Sep 2025 locked · Oct 2025 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 10:11am</t>
         </is>
       </c>
     </row>
@@ -6482,7 +7191,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Electrical &amp;&amp; Air Pty Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 job-margins.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:35am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 job-margins.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 10:11am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -6515,6 +7224,219 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Points for the target and break-even lines drawn on the charts (hidden sheet; edit the values on the chart's own sheet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Report: Job gross margin by type of job, October 2025: Target 35.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Report: Job gross margin by type of job, October 2025: Break-even 52.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Report: Job gross margin on each maintenance contract, October 2025: Target 35.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Report: Job gross margin on each maintenance contract, October 2025: Break-even 52.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Report: Job gross margin on each installation invoiced in October 2025: Target 35.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Report: Job gross margin on each installation invoiced in October 2025: Break-even 52.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Report: Job gross margin on call-outs by length, October 2025: Target 35.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Report: Job gross margin on call-outs by length, October 2025: Break-even 52.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G57"/>
@@ -6546,7 +7468,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Period: October 2025 · Data status: Sep 2025 locked · Oct 2025 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:35am</t>
+          <t>Period: October 2025 · Data status: Sep 2025 locked · Oct 2025 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 10:11am</t>
         </is>
       </c>
     </row>
@@ -8206,7 +9128,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Electrical &amp;&amp; Air Pty Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 job-margins.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:35am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 job-margins.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 10:11am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>